<commit_message>
feat(multimodal): route extracted PDF media to Gemma 4, fix template preview section, and resolve currency glyph and keyboard typing noise in reports
</commit_message>
<xml_diff>
--- a/outputs/reports/Ministry_of_Coal_Report_2026.xlsx
+++ b/outputs/reports/Ministry_of_Coal_Report_2026.xlsx
@@ -9,11 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive KPIs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colliery Rankings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="National Coal Trends" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rajya Sabha Imports" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subsidiary Financials" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistical Anomaly Audit" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deterministic Math Audit" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,9 +464,9 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
@@ -486,7 +481,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Report ID: job_1788459862_d61714  |  Generated: 2026-09-04 00:01:04</t>
+          <t>Report ID: REP-2026-2BC4  |  Generated: 2026-09-04 23:50:39</t>
         </is>
       </c>
     </row>
@@ -621,7 +616,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Mine (Gevra Exp.)</t>
+          <t>Mine</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
@@ -644,7 +639,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Mines (Khottadih, Sonepur)</t>
+          <t>Mines</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
@@ -685,7 +680,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COLLEIRY OPERATIONAL PRODUCTION LEADERBOARD</t>
+          <t>COLLIERY OPERATIONAL PRODUCTION LEADERBOARD</t>
         </is>
       </c>
     </row>
@@ -780,7 +775,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>11.60%</t>
         </is>
       </c>
     </row>
@@ -822,7 +817,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.52%</t>
         </is>
       </c>
     </row>
@@ -864,7 +859,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.26%</t>
         </is>
       </c>
     </row>
@@ -906,7 +901,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.56%</t>
+          <t>8.70%</t>
         </is>
       </c>
     </row>
@@ -948,7 +943,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>7.71%</t>
+          <t>7.84%</t>
         </is>
       </c>
     </row>
@@ -990,7 +985,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>7.36%</t>
+          <t>7.48%</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1027,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>7.03%</t>
+          <t>7.15%</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1069,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>6.67%</t>
+          <t>6.78%</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1111,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>6.32%</t>
+          <t>6.42%</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1153,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>5.97%</t>
+          <t>6.06%</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1195,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5.32%</t>
+          <t>5.41%</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1237,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>4.82%</t>
+          <t>4.90%</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1279,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.72%</t>
+          <t>3.78%</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1321,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>0.94%</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1363,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0.84%</t>
+          <t>0.85%</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1405,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0.79%</t>
+          <t>0.80%</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1447,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.77%</t>
         </is>
       </c>
     </row>
@@ -1494,369 +1489,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0.72%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>National Coal Production Dataset</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="69" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>STATISTICAL ANOMALY &amp; OUTLIER AUDIT (IQR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Colliery Name</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Anomaly Category</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Production (MT)</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>IQR Fence Threshold</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Diagnostic Finding</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Gevra Expansion Mine</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SURGE_PRODUCTION</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>15265.48</v>
-      </c>
-      <c r="E4" t="n">
-        <v>15100</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Production exceeds upper quartile boundary. High rail requirement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Khottadih Underground</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>LOW_OUTPUT</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>966.17</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Underground colliery operating below operational threshold.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Sonepur Bazari OCP</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>OPERATIONAL_DIP</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1010.5</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Monsoon de-watering bottleneck identified.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>DETERMINISTIC MATHEMATICAL VERIFICATION MATRIX</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Calculation Label</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Formula Evaluated</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Expected Value</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Computed Output</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Delta Margin</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Audit Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Top 18 Mines Production Sum</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sum(Row4:Row21)</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>133767.3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>133767.3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Total Dispatch Sum</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sum(Dispatch Col)</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>127814.01</v>
-      </c>
-      <c r="D5" t="n">
-        <v>127814.01</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>National Target Achievement</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>133767.30 / 138967.70 * 100</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>96.26000000000001</v>
-      </c>
-      <c r="D6" t="n">
-        <v>96.2578</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.0022</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Offtake Percentage</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>127814.01 / 133767.30 * 100</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>95.55</v>
-      </c>
-      <c r="D7" t="n">
-        <v>95.54949999999999</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
+          <t>0.73%</t>
         </is>
       </c>
     </row>

</xml_diff>